<commit_message>
Pivot export: shipment mode from bill keywords; drop cost per CBM
- Shipment mode is decided per invoice: FCL or container-type words mean
  FCL, CFS/CBM/LCL words mean LCL (FCL wins), else the volume format
- Remove the cost-per-CBM calculated field from KPI and unit-cost pivots

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/expense_dashboard/templates/pivot_template.xlsx
+++ b/expense_dashboard/templates/pivot_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\資誠claude code專案資料夾\invoice_excel_mapping\expense_dashboard\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9F9F94D-C939-4785-B8C2-7C59CDEE48B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{87FBD4DE-AF02-46ED-99B1-9E511964941A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15465" yWindow="-13620" windowWidth="24240" windowHeight="13020" xr2:uid="{2573DD42-5528-4BE5-8CB9-540C2F60DDE8}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="14400" windowHeight="8250" xr2:uid="{B1ED41E5-B6B8-4D84-ADBB-5CAC90EBF1FF}"/>
   </bookViews>
   <sheets>
     <sheet name="儀表板_總覽" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="24" r:id="rId15"/>
+    <pivotCache cacheId="23" r:id="rId15"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="77">
   <si>
     <t>INVOICE DATE 發票日期</t>
   </si>
@@ -227,9 +227,6 @@
     <t>每 TEU 成本 (USD)</t>
   </si>
   <si>
-    <t>每 CBM 成本 (USD)</t>
-  </si>
-  <si>
     <t>每月 × 費用大類 (USD)</t>
   </si>
   <si>
@@ -275,7 +272,7 @@
     <t>45HC</t>
   </si>
   <si>
-    <t>單位成本 (供應商)：每 TEU = FCL 費用 / TEU，每 CBM = LCL 費用 / CBM</t>
+    <t>單位成本 (供應商)：每 TEU 成本 = FCL 費用 / TEU</t>
   </si>
   <si>
     <t>FCL 費用</t>
@@ -695,7 +692,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-A628-4260-B7DC-9BA4B2BA9E1D}"/>
+              <c16:uniqueId val="{00000001-8623-4131-94D1-CC8B51B90094}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -709,11 +706,11 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="449671504"/>
-        <c:axId val="449672464"/>
+        <c:axId val="674074896"/>
+        <c:axId val="674075856"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="449671504"/>
+        <c:axId val="674074896"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -756,7 +753,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="449672464"/>
+        <c:crossAx val="674075856"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -764,7 +761,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="449672464"/>
+        <c:axId val="674075856"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -815,7 +812,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="449671504"/>
+        <c:crossAx val="674074896"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1086,7 +1083,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-FD59-4D3C-83FD-40873E6743F3}"/>
+              <c16:uniqueId val="{00000001-984E-4F93-970C-E18CD882E6E4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1099,11 +1096,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="449667664"/>
-        <c:axId val="449671024"/>
+        <c:axId val="1027693056"/>
+        <c:axId val="1027694016"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="449667664"/>
+        <c:axId val="1027693056"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1146,7 +1143,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="449671024"/>
+        <c:crossAx val="1027694016"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1154,7 +1151,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="449671024"/>
+        <c:axId val="1027694016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1205,7 +1202,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="449667664"/>
+        <c:crossAx val="1027693056"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1473,7 +1470,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-16D9-4472-8C6C-DAA4FF5C3977}"/>
+              <c16:uniqueId val="{00000001-010B-4921-9094-23CB4E67B6D3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1487,11 +1484,11 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="449671984"/>
-        <c:axId val="449672944"/>
+        <c:axId val="1027693536"/>
+        <c:axId val="1027694496"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="449671984"/>
+        <c:axId val="1027693536"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1534,7 +1531,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="449672944"/>
+        <c:crossAx val="1027694496"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1542,7 +1539,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="449672944"/>
+        <c:axId val="1027694496"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1593,7 +1590,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="449671984"/>
+        <c:crossAx val="1027693536"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1862,7 +1859,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-52BF-4946-8934-AF0DC5CEFBEE}"/>
+              <c16:uniqueId val="{00000001-21C4-4159-A8F6-228D692749E4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1876,11 +1873,11 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="449669104"/>
-        <c:axId val="449673904"/>
+        <c:axId val="1030306000"/>
+        <c:axId val="1030305520"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="449669104"/>
+        <c:axId val="1030306000"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1923,7 +1920,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="449673904"/>
+        <c:crossAx val="1030305520"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1931,7 +1928,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="449673904"/>
+        <c:axId val="1030305520"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1982,7 +1979,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="449669104"/>
+        <c:crossAx val="1030306000"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2407,7 +2404,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-0506-4FCE-8E87-E08476429540}"/>
+              <c16:uniqueId val="{00000001-BFEE-47BB-AE56-BF77AB52ED8B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2460,7 +2457,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-0506-4FCE-8E87-E08476429540}"/>
+              <c16:uniqueId val="{00000002-BFEE-47BB-AE56-BF77AB52ED8B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2513,7 +2510,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-0506-4FCE-8E87-E08476429540}"/>
+              <c16:uniqueId val="{00000003-BFEE-47BB-AE56-BF77AB52ED8B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2566,7 +2563,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-0506-4FCE-8E87-E08476429540}"/>
+              <c16:uniqueId val="{00000004-BFEE-47BB-AE56-BF77AB52ED8B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2580,11 +2577,11 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="451308528"/>
-        <c:axId val="451304688"/>
+        <c:axId val="1030306480"/>
+        <c:axId val="1030304080"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="451308528"/>
+        <c:axId val="1030306480"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2627,7 +2624,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="451304688"/>
+        <c:crossAx val="1030304080"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2635,7 +2632,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="451304688"/>
+        <c:axId val="1030304080"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2686,7 +2683,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="451308528"/>
+        <c:crossAx val="1030306480"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2955,7 +2952,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4126-483E-8ABA-9878AEA140FE}"/>
+              <c16:uniqueId val="{00000001-43F0-42D5-B5F5-20D09BAF88CD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2968,11 +2965,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="182"/>
-        <c:axId val="451302768"/>
-        <c:axId val="451306128"/>
+        <c:axId val="1030416752"/>
+        <c:axId val="1030417232"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="451302768"/>
+        <c:axId val="1030416752"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3015,7 +3012,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="451306128"/>
+        <c:crossAx val="1030417232"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3023,7 +3020,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="451306128"/>
+        <c:axId val="1030417232"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3074,7 +3071,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="451302768"/>
+        <c:crossAx val="1030416752"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3343,7 +3340,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-35CF-4DF1-9C43-DCB9D8913420}"/>
+              <c16:uniqueId val="{00000001-5982-4524-8D7D-BBCF0D8E78D8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3357,11 +3354,11 @@
         </c:dLbls>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="451304208"/>
-        <c:axId val="451307088"/>
+        <c:axId val="1030594944"/>
+        <c:axId val="1030593504"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="451304208"/>
+        <c:axId val="1030594944"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3404,7 +3401,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="451307088"/>
+        <c:crossAx val="1030593504"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3412,7 +3409,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="451307088"/>
+        <c:axId val="1030593504"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3463,7 +3460,7 @@
             <a:endParaRPr lang="zh-TW"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="451304208"/>
+        <c:crossAx val="1030594944"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7363,16 +7360,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>939800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>190497</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>79372</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
@@ -7381,7 +7378,7 @@
             <xdr:cNvPr id="2" name="國家">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F05E6B7-4F6C-D798-11D0-A550272068E5}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7C4F7E3-F934-42C0-A35F-F3926795E16D}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -7408,8 +7405,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6597650" y="2292350"/>
-              <a:ext cx="1828800" cy="2336797"/>
+              <a:off x="3486150" y="825500"/>
+              <a:ext cx="1828800" cy="2333622"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7441,16 +7438,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>939800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>190497</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>79372</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
@@ -7459,7 +7456,7 @@
             <xdr:cNvPr id="3" name="SUPPLIER 供應商名稱">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3EBF1249-1F28-158C-71F1-3D808C903872}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{723C57D3-1451-5411-0345-1E405F83561D}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -7486,8 +7483,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6597650" y="2292350"/>
-              <a:ext cx="1828800" cy="2336797"/>
+              <a:off x="3486150" y="825500"/>
+              <a:ext cx="1828800" cy="2333622"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7519,16 +7516,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>939800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>190497</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>79372</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
@@ -7537,7 +7534,7 @@
             <xdr:cNvPr id="4" name="年">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DD5BEF47-50A2-0145-B1B9-12026E161CC5}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{70B76759-BDAB-D4B1-1CBE-DC311B41F46C}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -7564,8 +7561,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6597650" y="2292350"/>
-              <a:ext cx="1828800" cy="2336797"/>
+              <a:off x="3486150" y="825500"/>
+              <a:ext cx="1828800" cy="2333622"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7597,16 +7594,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>939800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>190497</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>79372</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
@@ -7615,7 +7612,7 @@
             <xdr:cNvPr id="5" name="費用大類">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3FABA66A-E3DD-8254-7E91-7C1F49DA0AF3}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E79069B0-8FC0-03DA-EFAD-40D54A7FBCBA}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -7642,8 +7639,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6597650" y="2292350"/>
-              <a:ext cx="1828800" cy="2336797"/>
+              <a:off x="3486150" y="825500"/>
+              <a:ext cx="1828800" cy="2333622"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7676,22 +7673,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>206375</xdr:rowOff>
+      <xdr:colOff>127000</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>161925</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>273050</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>107950</xdr:rowOff>
+      <xdr:rowOff>209550</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="6" name="圖表 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1800119B-3544-96BC-3787-3CB88ED7F960}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AB1560A-DAD6-D3A1-8370-BC61F497F796}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7711,23 +7708,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>206375</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>180975</xdr:colOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>298450</xdr:colOff>
       <xdr:row>32</xdr:row>
-      <xdr:rowOff>107950</xdr:rowOff>
+      <xdr:rowOff>209550</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="7" name="圖表 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5FF58B2E-F345-9860-7B62-E86C8BB41DB3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F14A9801-940C-8BB5-BA9C-CEA24A1B9577}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7748,22 +7745,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
+      <xdr:colOff>127000</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>15875</xdr:rowOff>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>161925</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>136525</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>273050</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>82550</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="8" name="圖表 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{392793D5-4B66-8115-E111-C17CBBE67BF8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{99196CB6-DB60-8898-F07A-E5FD06CE46BD}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7783,23 +7780,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>15875</xdr:rowOff>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>180975</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>136525</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>298450</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>82550</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="9" name="圖表 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CAA60F51-3035-B823-98BC-B39CE8D58A21}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AAE664ED-D649-BF2C-021D-0652B52CC3C6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7824,16 +7821,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>504825</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>504825</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>190497</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>79372</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
@@ -7842,7 +7839,7 @@
             <xdr:cNvPr id="2" name="國家 1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{03B46CDE-A4A5-247D-6411-D8387B7D5D85}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D6F6C72-89BC-C5D0-94E6-8B197099B8EE}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -7869,8 +7866,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6597650" y="2292350"/>
-              <a:ext cx="1828800" cy="2336797"/>
+              <a:off x="3486150" y="825500"/>
+              <a:ext cx="1828800" cy="2333622"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7902,16 +7899,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>504825</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>504825</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>190497</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>79372</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
@@ -7920,7 +7917,7 @@
             <xdr:cNvPr id="3" name="SUPPLIER 供應商名稱 1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8320BE77-99F4-B19A-E887-89F5A021FAD9}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A573EF15-2615-EDFD-CAAB-BA3A0440A90D}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -7947,8 +7944,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6597650" y="2292350"/>
-              <a:ext cx="1828800" cy="2336797"/>
+              <a:off x="3486150" y="825500"/>
+              <a:ext cx="1828800" cy="2333622"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7980,16 +7977,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>504825</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>504825</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>190497</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>79372</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
@@ -7998,7 +7995,7 @@
             <xdr:cNvPr id="4" name="年 1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CB6895C0-FE06-A2AC-56C4-62B791C9E935}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AE252631-4882-2DBA-7251-5D4344287141}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -8025,8 +8022,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6597650" y="2292350"/>
-              <a:ext cx="1828800" cy="2336797"/>
+              <a:off x="3486150" y="825500"/>
+              <a:ext cx="1828800" cy="2333622"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -8058,16 +8055,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>504825</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>504825</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>190497</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>79372</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
@@ -8076,7 +8073,7 @@
             <xdr:cNvPr id="5" name="費用大類 1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF2E75C2-19FB-364A-DEF7-B04213492AF1}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7EDC8CDC-2125-9EF3-538B-13D781BFB58E}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -8103,8 +8100,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6597650" y="2292350"/>
-              <a:ext cx="1828800" cy="2336797"/>
+              <a:off x="3486150" y="825500"/>
+              <a:ext cx="1828800" cy="2333622"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -8137,22 +8134,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
+      <xdr:colOff>127000</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
+      <xdr:rowOff>196850</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
+      <xdr:colOff>25400</xdr:colOff>
       <xdr:row>29</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:rowOff>158750</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="6" name="圖表 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C686782D-D613-6326-BC7D-0DD65ECD041D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E379D500-61C7-D8E2-3743-2569CD0141BA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8175,20 +8172,20 @@
       <xdr:col>11</xdr:col>
       <xdr:colOff>152400</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
+      <xdr:rowOff>196850</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
+      <xdr:colOff>50800</xdr:colOff>
       <xdr:row>29</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
+      <xdr:rowOff>158750</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="7" name="圖表 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B61F53FA-1335-2852-4BD5-43B8D9CB6815}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6886A44F-77A9-793A-488B-9A4E6C40758F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8209,22 +8206,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>193675</xdr:rowOff>
+      <xdr:colOff>127000</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>69850</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="8" name="圖表 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{922764A3-0828-E8A8-4207-1A675C8FFD63}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43BCC219-213B-1053-DE75-E33CC555D87E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8246,11 +8243,11 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="" refreshedDate="46322.714291782409" missingItemsLimit="0" createdVersion="5" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2116379A-D551-4788-BFB1-F68BB7109533}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="" refreshedDate="46322.77512395833" missingItemsLimit="0" createdVersion="5" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{D7BD60B3-608F-462F-9C70-C8E8018E3F92}">
   <cacheSource type="worksheet">
     <worksheetSource name="明細表"/>
   </cacheSource>
-  <cacheFields count="45">
+  <cacheFields count="44">
     <cacheField name="INVOICE DATE 發票日期" numFmtId="176">
       <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-01-01T00:00:00" maxDate="2026-01-02T00:00:00"/>
     </cacheField>
@@ -8397,20 +8394,19 @@
       <sharedItems/>
     </cacheField>
     <cacheField name="每TEU成本" numFmtId="0" formula="'FCL 費用 (USD)'/TEU" databaseField="0"/>
-    <cacheField name="每CBM成本" numFmtId="0" formula="'LCL 費用 (USD)'/CBM" databaseField="0"/>
   </cacheFields>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition pivotCacheId="341430193"/>
+      <x14:pivotCacheDefinition pivotCacheId="1513859983"/>
     </ext>
   </extLst>
 </pivotCacheDefinition>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{59441AF4-8125-40B3-AB76-EFEC9D6613C4}" name="PT_KPI" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A4:F5" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="45">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CA7B781B-5EB8-458D-876A-C20DCAE10F3A}" name="PT_KPI" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A4:E5" firstHeaderRow="0" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="44">
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
@@ -8475,7 +8471,6 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField dataField="1" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField dataField="1" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowItems count="1">
     <i/>
@@ -8483,7 +8478,7 @@
   <colFields count="1">
     <field x="-2"/>
   </colFields>
-  <colItems count="6">
+  <colItems count="5">
     <i>
       <x/>
     </i>
@@ -8499,17 +8494,13 @@
     <i i="4">
       <x v="4"/>
     </i>
-    <i i="5">
-      <x v="5"/>
-    </i>
   </colItems>
-  <dataFields count="6">
+  <dataFields count="5">
     <dataField name="USD 金額" fld="20" baseField="0" baseItem="0" numFmtId="4"/>
     <dataField name="發票數" fld="40" baseField="0" baseItem="0" numFmtId="3"/>
     <dataField name="TEU 數" fld="35" baseField="0" baseItem="0" numFmtId="3"/>
     <dataField name="CBM 數" fld="36" baseField="0" baseItem="0" numFmtId="178"/>
     <dataField name="每 TEU 成本 (USD)" fld="43" baseField="0" baseItem="0" numFmtId="4"/>
-    <dataField name="每 CBM 成本 (USD)" fld="44" baseField="0" baseItem="0" numFmtId="4"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -8524,9 +8515,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable10.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5DAA4AFA-A314-4EB1-B87A-1A30B3AC445C}" name="PT_單位成本_航線" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:G5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="45">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B4CC979A-20FB-46F6-843C-3EA4CD742EB6}" name="PT_單位成本_航線" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:F5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="44">
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
@@ -8604,7 +8595,6 @@
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField dataField="1" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dataField="1" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -8621,7 +8611,7 @@
   <colFields count="1">
     <field x="-2"/>
   </colFields>
-  <colItems count="6">
+  <colItems count="5">
     <i>
       <x/>
     </i>
@@ -8637,17 +8627,13 @@
     <i i="4">
       <x v="4"/>
     </i>
-    <i i="5">
-      <x v="5"/>
-    </i>
   </colItems>
-  <dataFields count="6">
+  <dataFields count="5">
     <dataField name="TEU 數" fld="35" baseField="0" baseItem="0" numFmtId="3"/>
     <dataField name="FCL 費用" fld="38" baseField="0" baseItem="0" numFmtId="4"/>
     <dataField name="每 TEU 成本 (USD)" fld="43" baseField="0" baseItem="0" numFmtId="4"/>
     <dataField name="LCL 費用" fld="39" baseField="0" baseItem="0" numFmtId="4"/>
     <dataField name="CBM 數" fld="36" baseField="0" baseItem="0" numFmtId="178"/>
-    <dataField name="每 CBM 成本 (USD)" fld="44" baseField="0" baseItem="0" numFmtId="4"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <filters count="1">
@@ -8671,9 +8657,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable11.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{70DDBC77-36D9-4F62-BB0B-F2342A2C38CB}" name="PT_航線" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{352D2B73-A9DB-49E0-AB45-5A8A01900519}" name="PT_航線" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A3:B5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="45">
+  <pivotFields count="44">
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
@@ -8751,7 +8737,6 @@
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -8804,9 +8789,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{74879E4B-480A-4C12-8C3E-7BAC3D533B66}" name="PT_每月費用大類" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{87320E55-0C94-498B-8782-8BE87F4BA99B}" name="PT_每月費用大類" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A3:C6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="45">
+  <pivotFields count="44">
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
@@ -8875,7 +8860,6 @@
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -8930,9 +8914,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EF9368FE-44FB-4A88-B132-5308202E4733}" name="PT_年度比較" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1B3B69AA-276D-4BD6-8CE8-FE0E882770BD}" name="PT_年度比較" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A3:C6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="45">
+  <pivotFields count="44">
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
@@ -9001,7 +8985,6 @@
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -9056,9 +9039,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DF1B6232-FF2D-4EE7-BD7D-E8805FFE5E60}" name="PT_供應商排名" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5D16DD49-0816-4F2B-B4AA-7E434CCE31B4}" name="PT_供應商排名" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:D5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="45">
+  <pivotFields count="44">
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0" sortType="descending">
@@ -9131,7 +9114,6 @@
     <pivotField dataField="1" numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -9177,9 +9159,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E8520181-2AA9-49B3-8BE3-010C13E278EF}" name="PT_供應商月份" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5002E066-63C2-42B0-8CCB-F73BA696CD41}" name="PT_供應商月份" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A3:C7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="45">
+  <pivotFields count="44">
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisCol" showAll="0">
@@ -9248,7 +9230,6 @@
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="2">
@@ -9307,9 +9288,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{79CE60CB-B5CC-47AF-ACA9-21415ABBEEC9}" name="PT_費用大類" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{20FC6816-DB04-4556-9F1E-541D42A45C12}" name="PT_費用大類" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A3:C6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="45">
+  <pivotFields count="44">
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisCol" showAll="0">
@@ -9382,7 +9363,6 @@
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -9437,9 +9417,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B92C70EA-5B5A-4B5B-8511-52393FE7A533}" name="PT_集團公司" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DBA43051-FB48-406A-85F6-8526F98CF406}" name="PT_集團公司" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A3:C6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="45">
+  <pivotFields count="44">
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
@@ -9517,7 +9497,6 @@
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -9572,9 +9551,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{37530A12-3C84-4342-8793-715D8BF9AA36}" name="PT_運量" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{55DF292A-7842-471D-B09B-DDBB9CB518EF}" name="PT_運量" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A3:E5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="45">
+  <pivotFields count="44">
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0">
@@ -9643,7 +9622,6 @@
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -9731,9 +9709,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{09538EE3-167C-43D0-B6EF-83A93C85EE91}" name="PT_單位成本_供應商" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:G5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="45">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{29FD5C92-FBC7-4E1A-8592-A8CAA1DBBCA7}" name="PT_單位成本_供應商" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" errorCaption="-" showError="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="1" itemPrintTitles="1" createdVersion="5" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:F5" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="44">
     <pivotField numFmtId="176" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0" sortType="descending">
@@ -9806,7 +9784,6 @@
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField dataField="1" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
     <pivotField dataField="1" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -9823,7 +9800,7 @@
   <colFields count="1">
     <field x="-2"/>
   </colFields>
-  <colItems count="6">
+  <colItems count="5">
     <i>
       <x/>
     </i>
@@ -9839,17 +9816,13 @@
     <i i="4">
       <x v="4"/>
     </i>
-    <i i="5">
-      <x v="5"/>
-    </i>
   </colItems>
-  <dataFields count="6">
+  <dataFields count="5">
     <dataField name="FCL 費用" fld="38" baseField="0" baseItem="0" numFmtId="4"/>
     <dataField name="TEU 數" fld="35" baseField="0" baseItem="0" numFmtId="3"/>
     <dataField name="每 TEU 成本 (USD)" fld="43" baseField="0" baseItem="0" numFmtId="4"/>
     <dataField name="LCL 費用" fld="39" baseField="0" baseItem="0" numFmtId="4"/>
     <dataField name="CBM 數" fld="36" baseField="0" baseItem="0" numFmtId="178"/>
-    <dataField name="每 CBM 成本 (USD)" fld="44" baseField="0" baseItem="0" numFmtId="4"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -9864,7 +9837,7 @@
 </file>
 
 <file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_國家" xr10:uid="{0C6924CD-8AA9-4635-9554-748C1AFD8971}" sourceName="國家">
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_國家" xr10:uid="{DE274A62-6C78-4660-8FA4-1100D84FD0AA}" sourceName="國家">
   <pivotTables>
     <pivotTable tabId="1" name="PT_KPI"/>
     <pivotTable tabId="4" name="PT_每月費用大類"/>
@@ -9879,7 +9852,7 @@
     <pivotTable tabId="13" name="PT_航線"/>
   </pivotTables>
   <data>
-    <tabular pivotCacheId="341430193">
+    <tabular pivotCacheId="1513859983">
       <items count="1">
         <i x="0" s="1"/>
       </items>
@@ -9889,7 +9862,7 @@
 </file>
 
 <file path=xl/slicerCaches/slicerCache2.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_SUPPLIER_供應商名稱" xr10:uid="{FF7C1E86-ABD8-40ED-927B-F83DD9827A05}" sourceName="SUPPLIER 供應商名稱">
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_SUPPLIER_供應商名稱" xr10:uid="{DEBCBBDB-3CF4-4EA7-9662-2F89E245E51D}" sourceName="SUPPLIER 供應商名稱">
   <pivotTables>
     <pivotTable tabId="1" name="PT_KPI"/>
     <pivotTable tabId="4" name="PT_每月費用大類"/>
@@ -9904,7 +9877,7 @@
     <pivotTable tabId="13" name="PT_航線"/>
   </pivotTables>
   <data>
-    <tabular pivotCacheId="341430193">
+    <tabular pivotCacheId="1513859983">
       <items count="1">
         <i x="0" s="1"/>
       </items>
@@ -9914,7 +9887,7 @@
 </file>
 
 <file path=xl/slicerCaches/slicerCache3.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_年" xr10:uid="{F2556E91-E61A-4BB2-BC63-CDBBF5385AFB}" sourceName="年">
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_年" xr10:uid="{B485A9CD-65D1-469B-880D-875078AC22C8}" sourceName="年">
   <pivotTables>
     <pivotTable tabId="1" name="PT_KPI"/>
     <pivotTable tabId="4" name="PT_每月費用大類"/>
@@ -9929,7 +9902,7 @@
     <pivotTable tabId="13" name="PT_航線"/>
   </pivotTables>
   <data>
-    <tabular pivotCacheId="341430193">
+    <tabular pivotCacheId="1513859983">
       <items count="1">
         <i x="0" s="1"/>
       </items>
@@ -9939,7 +9912,7 @@
 </file>
 
 <file path=xl/slicerCaches/slicerCache4.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_費用大類" xr10:uid="{D590E2D3-9E31-4AA7-88B3-D9194AC10CF4}" sourceName="費用大類">
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_費用大類" xr10:uid="{25431627-1E18-460B-AFED-5447F77CCC55}" sourceName="費用大類">
   <pivotTables>
     <pivotTable tabId="1" name="PT_KPI"/>
     <pivotTable tabId="4" name="PT_每月費用大類"/>
@@ -9954,7 +9927,7 @@
     <pivotTable tabId="13" name="PT_航線"/>
   </pivotTables>
   <data>
-    <tabular pivotCacheId="341430193">
+    <tabular pivotCacheId="1513859983">
       <items count="1">
         <i x="0" s="1"/>
       </items>
@@ -9965,80 +9938,80 @@
 
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="國家" xr10:uid="{6C0A8404-C2F8-42F6-A0D8-D97631E7AF5C}" cache="Slicer_國家" caption="國家" rowHeight="220133"/>
-  <slicer name="SUPPLIER 供應商名稱" xr10:uid="{3EC8ABB1-421E-4EBD-B770-4E091E13B5A6}" cache="Slicer_SUPPLIER_供應商名稱" caption="SUPPLIER 供應商名稱" rowHeight="220133"/>
-  <slicer name="年" xr10:uid="{9F12D052-DC10-416E-953D-CDD16B831657}" cache="Slicer_年" caption="年" rowHeight="220133"/>
-  <slicer name="費用大類" xr10:uid="{1804D4D9-A5A9-48CD-A28B-A817A42D98D7}" cache="Slicer_費用大類" caption="費用大類" rowHeight="220133"/>
+  <slicer name="國家" xr10:uid="{563069CA-F2B3-45E7-9AF6-1F4E8C9BB79E}" cache="Slicer_國家" caption="國家" rowHeight="220133"/>
+  <slicer name="SUPPLIER 供應商名稱" xr10:uid="{8AF8C9EA-A4BB-41E7-88C6-B5AF8F7119AE}" cache="Slicer_SUPPLIER_供應商名稱" caption="SUPPLIER 供應商名稱" rowHeight="220133"/>
+  <slicer name="年" xr10:uid="{2572516B-3823-4D0E-B717-EBF539C3A453}" cache="Slicer_年" caption="年" rowHeight="220133"/>
+  <slicer name="費用大類" xr10:uid="{D33DF2FE-78C0-4083-A03F-05640B5A2678}" cache="Slicer_費用大類" caption="費用大類" rowHeight="220133"/>
 </slicers>
 </file>
 
 <file path=xl/slicers/slicer2.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="國家 1" xr10:uid="{969B2AB5-429F-42A9-9902-307CD038B2DC}" cache="Slicer_國家" caption="國家" rowHeight="220133"/>
-  <slicer name="SUPPLIER 供應商名稱 1" xr10:uid="{AE1CD86A-2D57-4342-AD0D-552FB14B054D}" cache="Slicer_SUPPLIER_供應商名稱" caption="SUPPLIER 供應商名稱" rowHeight="220133"/>
-  <slicer name="年 1" xr10:uid="{1BCAE515-77E1-46CA-8EB2-722A022384D4}" cache="Slicer_年" caption="年" rowHeight="220133"/>
-  <slicer name="費用大類 1" xr10:uid="{4C065B2C-0853-40D9-944D-EB8FB1A19CA8}" cache="Slicer_費用大類" caption="費用大類" rowHeight="220133"/>
+  <slicer name="國家 1" xr10:uid="{9131DC52-1304-4539-8785-B95206DBB706}" cache="Slicer_國家" caption="國家" rowHeight="220133"/>
+  <slicer name="SUPPLIER 供應商名稱 1" xr10:uid="{9CF37B31-4866-4687-8CB7-8DDD8C90AFEB}" cache="Slicer_SUPPLIER_供應商名稱" caption="SUPPLIER 供應商名稱" rowHeight="220133"/>
+  <slicer name="年 1" xr10:uid="{C522B6CE-3538-4A1E-8C49-E4D7CC087B5F}" cache="Slicer_年" caption="年" rowHeight="220133"/>
+  <slicer name="費用大類 1" xr10:uid="{0007A081-F8CC-4DD2-9095-87A8E0F48137}" cache="Slicer_費用大類" caption="費用大類" rowHeight="220133"/>
 </slicers>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4F8FF43C-74BD-4E61-9AC8-FFC40299264F}" name="明細表" displayName="明細表" ref="A1:AQ2" totalsRowShown="0">
-  <autoFilter ref="A1:AQ2" xr:uid="{4F8FF43C-74BD-4E61-9AC8-FFC40299264F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{536E6309-83E0-4CC2-A4E0-7277AB1983C8}" name="明細表" displayName="明細表" ref="A1:AQ2" totalsRowShown="0">
+  <autoFilter ref="A1:AQ2" xr:uid="{536E6309-83E0-4CC2-A4E0-7277AB1983C8}"/>
   <tableColumns count="43">
-    <tableColumn id="1" xr3:uid="{A9CA7183-3A51-4D9A-AD4E-F97425C8DD54}" name="INVOICE DATE 發票日期" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{A31B069C-D97D-485B-BA8C-E136A4EAAD45}" name="INVOICE NO 發票號碼"/>
-    <tableColumn id="3" xr3:uid="{9593EB8D-EA49-41F9-8DB9-B83CF42C55F0}" name="SUPPLIER 供應商名稱"/>
-    <tableColumn id="4" xr3:uid="{F1349514-97BE-4435-85BD-0D3D1AFDFAA3}" name="CONSIGNEE 集團公司名稱"/>
-    <tableColumn id="5" xr3:uid="{41DE48B6-317A-49FC-9982-494100567D4B}" name="Description 費用名稱"/>
-    <tableColumn id="6" xr3:uid="{9ADBC217-8563-460C-8702-7C200E5A2433}" name="AMOUNT 金額" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{6B2CE3EE-ACED-44E4-B80F-DBF9EF15FCC4}" name="VAT 稅額" dataDxfId="17"/>
-    <tableColumn id="8" xr3:uid="{856A8678-707B-420E-BE51-60FE1887DAC6}" name="Order No."/>
-    <tableColumn id="9" xr3:uid="{C4DF4891-9C43-4724-9A25-59115F8C882C}" name="Arrive Date 到達日" dataDxfId="16"/>
-    <tableColumn id="10" xr3:uid="{E11077E5-5552-428A-A9CE-5350CFE1BE88}" name="on board date 開船日" dataDxfId="15"/>
-    <tableColumn id="11" xr3:uid="{C25CEAE0-B56C-407C-9B1F-CB6657FAEE2F}" name="B/L NO. 提單號碼"/>
-    <tableColumn id="12" xr3:uid="{937A83E5-4290-4403-A3C4-B3E249F535B9}" name="MBL NO. 主提單號碼"/>
-    <tableColumn id="13" xr3:uid="{CFDCAE64-3B3D-434B-83F4-9F9DBC1D6EE6}" name="Port of Loading 啟運港"/>
-    <tableColumn id="14" xr3:uid="{F818B2D5-C812-47A6-9419-DBC964C8A326}" name="Port of discharge 目的港"/>
-    <tableColumn id="15" xr3:uid="{9AB73CBD-A300-474E-B799-F2C6E8126B17}" name="Volume 材積"/>
-    <tableColumn id="16" xr3:uid="{1CDBE89E-123C-4D06-A8D3-8180AB65A4F7}" name="Vessel 船名"/>
-    <tableColumn id="17" xr3:uid="{1C137FDB-B7FF-481C-930A-63873DE21D35}" name="Container no. 貨櫃號碼"/>
-    <tableColumn id="18" xr3:uid="{D77E18E5-70F8-4FE4-9DE6-9177D86625F9}" name="Shipper 出貨方"/>
-    <tableColumn id="19" xr3:uid="{B0DF156C-54A7-415B-9312-4AEA4A93D01D}" name="原幣別"/>
-    <tableColumn id="20" xr3:uid="{C7EF7F4A-40A0-4411-A7CB-F8F26F9BAB04}" name="匯率 (1 USD = ?)" dataDxfId="14"/>
-    <tableColumn id="21" xr3:uid="{83DE1BF1-3FC9-4F57-8FDF-80799ECDFD72}" name="AMOUNT (USD)" dataDxfId="13"/>
-    <tableColumn id="22" xr3:uid="{C4C0A3F4-06C2-47A7-ACC8-E2260EF7D54A}" name="VAT (USD)" dataDxfId="12"/>
-    <tableColumn id="23" xr3:uid="{ED3FDCBA-48AF-4E10-A456-A6B78DC50164}" name="費用大類"/>
-    <tableColumn id="24" xr3:uid="{6DE1AB2C-9CE1-4F6D-AD92-203D5A225CC6}" name="費用項目 (標準化)"/>
-    <tableColumn id="25" xr3:uid="{9C54050F-E2E6-460D-A867-7FC03DDB35F4}" name="國家"/>
-    <tableColumn id="26" xr3:uid="{A4CEA04A-57E8-43D4-8EDA-3C59B04AD34C}" name="年" dataDxfId="11"/>
-    <tableColumn id="27" xr3:uid="{68E520B4-ADE0-4CC2-99A6-A357188AB4AA}" name="季"/>
-    <tableColumn id="28" xr3:uid="{A646C4D7-B49C-41CC-9240-894E081FC79C}" name="月" dataDxfId="10"/>
-    <tableColumn id="29" xr3:uid="{7FFCD647-F574-4529-8BC5-FFAA430AA45C}" name="年月"/>
-    <tableColumn id="30" xr3:uid="{E8F7F3C9-A920-421A-9AD8-C1D766AEFE41}" name="航線"/>
-    <tableColumn id="31" xr3:uid="{42630F62-ABDE-4CD7-BB01-BE881F7CA706}" name="運送型態"/>
-    <tableColumn id="32" xr3:uid="{3A55A369-A8CC-48B3-BDC7-CD5716CA3B30}" name="20GP 櫃數" dataDxfId="9"/>
-    <tableColumn id="33" xr3:uid="{7F0016BE-D59E-4149-B772-59C678F00E0A}" name="40GP 櫃數" dataDxfId="8"/>
-    <tableColumn id="34" xr3:uid="{9D3F1F7E-E738-4EE8-B81E-78C0FEB44731}" name="40HC 櫃數" dataDxfId="7"/>
-    <tableColumn id="35" xr3:uid="{499CCFC7-EFC7-41A8-9511-99AF44520708}" name="45HC 櫃數" dataDxfId="6"/>
-    <tableColumn id="36" xr3:uid="{B07CDFC0-658B-48A4-A9FF-C86F0280A22C}" name="TEU" dataDxfId="5"/>
-    <tableColumn id="37" xr3:uid="{856E1CF9-DCDC-4F59-BBF4-43D01AC04A73}" name="CBM" dataDxfId="4"/>
-    <tableColumn id="38" xr3:uid="{7987076F-EB2C-4D3F-B94A-9FDA7D706C1E}" name="重量 KG" dataDxfId="3"/>
-    <tableColumn id="39" xr3:uid="{8EE9B9A8-49C7-4F8B-8D3F-18D4F763123C}" name="FCL 費用 (USD)" dataDxfId="2"/>
-    <tableColumn id="40" xr3:uid="{7524FC64-5F5B-4903-8995-11356D0102C3}" name="LCL 費用 (USD)" dataDxfId="1"/>
-    <tableColumn id="41" xr3:uid="{4B66E724-123C-4C61-949F-83B7D1823F96}" name="發票張數" dataDxfId="0"/>
-    <tableColumn id="42" xr3:uid="{1EE16B36-BFA7-4D26-BA5A-527B2875D63B}" name="來源資料夾"/>
-    <tableColumn id="43" xr3:uid="{97995065-B6F9-42BC-931A-0E4F785F6DA9}" name="來源檔案"/>
+    <tableColumn id="1" xr3:uid="{2279D1C9-56E6-42C2-A434-BD0015374A19}" name="INVOICE DATE 發票日期" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{6054866D-C469-4E79-8C74-B228A39AD5C2}" name="INVOICE NO 發票號碼"/>
+    <tableColumn id="3" xr3:uid="{D61CADDC-36E3-4951-9C18-171BDC55C930}" name="SUPPLIER 供應商名稱"/>
+    <tableColumn id="4" xr3:uid="{A1383D81-E9E1-4F26-8B55-106FB0CD5366}" name="CONSIGNEE 集團公司名稱"/>
+    <tableColumn id="5" xr3:uid="{359BFFE8-CA97-46E5-83A4-5FAB4D1FE3F3}" name="Description 費用名稱"/>
+    <tableColumn id="6" xr3:uid="{304CC7A2-2644-41E3-A479-2DC977672A68}" name="AMOUNT 金額" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{EE55F3C8-B2F5-4C7E-B946-5293B9A1A5B0}" name="VAT 稅額" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{F4DA8F10-3B94-4F06-B4AD-01E367E16D55}" name="Order No."/>
+    <tableColumn id="9" xr3:uid="{48DC066F-626A-4421-8C91-4467848E7325}" name="Arrive Date 到達日" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{C9CCBD70-2EAD-4451-A487-463167C631D3}" name="on board date 開船日" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{C1EB9BF5-7D87-4501-891C-A6B9987FB667}" name="B/L NO. 提單號碼"/>
+    <tableColumn id="12" xr3:uid="{01886B00-D230-4B8A-B50E-CD5EED3D447F}" name="MBL NO. 主提單號碼"/>
+    <tableColumn id="13" xr3:uid="{02C098A7-6C68-4A1B-AF57-6013B20C39EC}" name="Port of Loading 啟運港"/>
+    <tableColumn id="14" xr3:uid="{B631DC02-35F6-48D3-AFC8-9F35124A67B4}" name="Port of discharge 目的港"/>
+    <tableColumn id="15" xr3:uid="{962A8104-C93C-4CB5-BF51-66B7AD414D8A}" name="Volume 材積"/>
+    <tableColumn id="16" xr3:uid="{8C92A904-5829-4AA1-886A-A2AF5762C400}" name="Vessel 船名"/>
+    <tableColumn id="17" xr3:uid="{0F6CC08A-58F1-4DE7-8FD3-2088C06159E8}" name="Container no. 貨櫃號碼"/>
+    <tableColumn id="18" xr3:uid="{D2CBB456-A5B4-4845-B597-F40B2E6E28FD}" name="Shipper 出貨方"/>
+    <tableColumn id="19" xr3:uid="{CF72DC69-6EEF-45CD-B04A-8264832AC232}" name="原幣別"/>
+    <tableColumn id="20" xr3:uid="{6F14B261-4022-4E4E-B655-ED2B683C8C52}" name="匯率 (1 USD = ?)" dataDxfId="14"/>
+    <tableColumn id="21" xr3:uid="{C5218551-411C-44DD-AE17-14C231D3E7B8}" name="AMOUNT (USD)" dataDxfId="13"/>
+    <tableColumn id="22" xr3:uid="{94F5E505-4CF5-4ECE-B734-372CB4C1DBEF}" name="VAT (USD)" dataDxfId="12"/>
+    <tableColumn id="23" xr3:uid="{4BB2868C-1154-4BAB-AEDD-FBD5B002079E}" name="費用大類"/>
+    <tableColumn id="24" xr3:uid="{5207E985-1F39-4D72-8DEB-2028B5B1C776}" name="費用項目 (標準化)"/>
+    <tableColumn id="25" xr3:uid="{73A91353-2C12-443C-84FC-E58A83587CCD}" name="國家"/>
+    <tableColumn id="26" xr3:uid="{342984DB-E9B9-49B1-9AA7-B745A8DD6122}" name="年" dataDxfId="11"/>
+    <tableColumn id="27" xr3:uid="{3FAB2159-E8ED-4D5D-B5C4-60B14CB4C4C9}" name="季"/>
+    <tableColumn id="28" xr3:uid="{4D72578A-EA6F-4EEB-8676-EA4F90882A7C}" name="月" dataDxfId="10"/>
+    <tableColumn id="29" xr3:uid="{2849F91A-B281-44CC-BE72-644BCEC1DBC6}" name="年月"/>
+    <tableColumn id="30" xr3:uid="{3947412B-C7CA-409A-A11A-0D7D50404917}" name="航線"/>
+    <tableColumn id="31" xr3:uid="{5D5BC8AC-0D57-44A2-95F8-B13CF46825DF}" name="運送型態"/>
+    <tableColumn id="32" xr3:uid="{01EAF0EF-FF37-4FB9-B13E-94BFC230FED8}" name="20GP 櫃數" dataDxfId="9"/>
+    <tableColumn id="33" xr3:uid="{4DE83C2E-A5D7-4502-908B-A7E5214971FF}" name="40GP 櫃數" dataDxfId="8"/>
+    <tableColumn id="34" xr3:uid="{3421175F-0DC6-4805-BFE3-F465D8751F10}" name="40HC 櫃數" dataDxfId="7"/>
+    <tableColumn id="35" xr3:uid="{8346C7F4-D522-43F8-A9F2-8B93C7CF74A4}" name="45HC 櫃數" dataDxfId="6"/>
+    <tableColumn id="36" xr3:uid="{1EA2CE0B-B5D0-49E7-858C-B56F1BEA5EB5}" name="TEU" dataDxfId="5"/>
+    <tableColumn id="37" xr3:uid="{05F6FC02-301A-4D43-B974-C2C1101ED33B}" name="CBM" dataDxfId="4"/>
+    <tableColumn id="38" xr3:uid="{7A5B4FC9-53C8-4985-B003-DDA293C25089}" name="重量 KG" dataDxfId="3"/>
+    <tableColumn id="39" xr3:uid="{8980DEB9-3DB4-464D-93B0-29B8CB4BE6EF}" name="FCL 費用 (USD)" dataDxfId="2"/>
+    <tableColumn id="40" xr3:uid="{48F30DED-4705-49A1-9255-BC63EE6B8AC0}" name="LCL 費用 (USD)" dataDxfId="1"/>
+    <tableColumn id="41" xr3:uid="{6297C168-D8BF-4970-88EB-4114662E20D1}" name="發票張數" dataDxfId="0"/>
+    <tableColumn id="42" xr3:uid="{F9300900-E87B-4A2A-B89A-86469DD712A5}" name="來源資料夾"/>
+    <tableColumn id="43" xr3:uid="{C29235AA-C97D-47FF-BD39-5DA44CD5F4E8}" name="來源檔案"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2A8F817F-B4CF-4ACA-A96A-0F1C860BAA4C}" name="讀取失敗表" displayName="讀取失敗表" ref="A1:B2" totalsRowShown="0">
-  <autoFilter ref="A1:B2" xr:uid="{2A8F817F-B4CF-4ACA-A96A-0F1C860BAA4C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B19D9851-E119-4639-955E-9DC179B82AFF}" name="讀取失敗表" displayName="讀取失敗表" ref="A1:B2" totalsRowShown="0">
+  <autoFilter ref="A1:B2" xr:uid="{B19D9851-E119-4639-955E-9DC179B82AFF}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{FDAE397B-B2A2-44D1-8E2F-CE32E53BD2C5}" name="檔案"/>
-    <tableColumn id="2" xr3:uid="{7F47CB50-A78D-4941-AF88-DF8D13E0DD9E}" name="原因"/>
+    <tableColumn id="1" xr3:uid="{ADAB04E6-A735-47D8-837B-578A113B2493}" name="檔案"/>
+    <tableColumn id="2" xr3:uid="{D3F91ED5-1226-438F-A188-D27B80D7C4E7}" name="原因"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -10360,29 +10333,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39557176-3840-4E1D-A1DC-4632C2405308}">
-  <dimension ref="A1:F5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15405D6F-41B9-4037-A093-0C57789F5121}">
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21.5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="21.5" x14ac:dyDescent="0.4">
       <c r="A1" s="13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -10398,11 +10370,8 @@
       <c r="E4" t="s">
         <v>50</v>
       </c>
-      <c r="F4" t="s">
-        <v>51</v>
-      </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>0</v>
       </c>
@@ -10416,9 +10385,6 @@
         <v>0</v>
       </c>
       <c r="E5" s="2">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -10437,30 +10403,29 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68DBDB70-5572-4EF9-A6D7-E091B496893C}">
-  <dimension ref="A1:G5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAA470CB-3F0D-4839-B6B0-A48D52B92490}">
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A3" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" t="s">
         <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A3" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" t="s">
-        <v>68</v>
       </c>
       <c r="C3" t="s">
         <v>48</v>
@@ -10469,16 +10434,13 @@
         <v>50</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F3" t="s">
         <v>49</v>
       </c>
-      <c r="G3" t="s">
-        <v>51</v>
-      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="9" t="s">
         <v>43</v>
       </c>
@@ -10497,13 +10459,10 @@
       <c r="F4" s="6">
         <v>0</v>
       </c>
-      <c r="G4" s="2">
-        <v>0</v>
-      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" s="2">
         <v>0</v>
@@ -10518,9 +10477,6 @@
         <v>0</v>
       </c>
       <c r="F5" s="6">
-        <v>0</v>
-      </c>
-      <c r="G5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -10531,48 +10487,44 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11B1CF52-BA00-49BE-A1A5-6ACF8EF6B355}">
-  <dimension ref="A1:G5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E69E414-6E1C-44FD-8864-17AD0406113A}">
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="19.5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
         <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D3" t="s">
         <v>50</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F3" t="s">
         <v>49</v>
       </c>
-      <c r="G3" t="s">
-        <v>51</v>
-      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="9" t="s">
         <v>43</v>
       </c>
@@ -10591,13 +10543,10 @@
       <c r="F4" s="6">
         <v>0</v>
       </c>
-      <c r="G4" s="2">
-        <v>0</v>
-      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" s="5">
         <v>0</v>
@@ -10612,9 +10561,6 @@
         <v>0</v>
       </c>
       <c r="F5" s="6">
-        <v>0</v>
-      </c>
-      <c r="G5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -10625,22 +10571,22 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8CEE2C0-69FA-4ABA-9E33-33E2A318D707}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52BB783D-AD97-49CC-AB3E-57243D0E3D91}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
         <v>46</v>
@@ -10656,7 +10602,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" s="2">
         <v>0</v>
@@ -10669,7 +10615,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD900A9-5DA0-4092-92F8-A1CDCAD84FB5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68AD313F-9B41-4601-A883-2533F6A41B07}">
   <dimension ref="A1:AQ2"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
@@ -10972,7 +10918,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF88AADA-2DC3-4965-92F6-06BB5297C9BA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1945BE6-8D2A-44CF-8A68-BD52550E8025}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
@@ -10981,18 +10927,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" t="s">
         <v>72</v>
-      </c>
-      <c r="B1" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -11005,18 +10951,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16F87E89-B9D6-496B-833D-C4E6D93FCFEA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70E9ABA6-64AA-48D2-9A82-AF0394E2B244}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:1" ht="21.5" x14ac:dyDescent="0.4">
       <c r="A1" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -11034,18 +10980,18 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7911282-98EC-4747-A8C0-ED1C0EC2A384}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F305367-F9DB-44BB-ACC8-6A5005BC6A8D}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.4">
@@ -11053,18 +10999,18 @@
         <v>46</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
         <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
@@ -11080,7 +11026,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" s="2">
         <v>0</v>
@@ -11096,18 +11042,18 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{184EBCD5-6D98-4673-9274-0916EEDF1A04}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82802975-9AC7-4CB3-AC2A-59AB1667A2FA}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.4">
@@ -11115,18 +11061,18 @@
         <v>46</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B4" s="4">
         <v>2026</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
@@ -11142,7 +11088,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" s="2">
         <v>0</v>
@@ -11158,30 +11104,30 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F86EBA47-545B-459D-9CEC-4DDF1339D2AD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BF9CA93-B243-4597-AD43-7C5C6141D5A1}">
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
         <v>46</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D3" t="s">
         <v>47</v>
@@ -11203,7 +11149,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" s="2">
         <v>0</v>
@@ -11222,18 +11168,18 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{601CF029-841A-4281-A37A-DC79821D26E5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53C099AB-4CDA-4258-B0A1-0658DC495F61}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.4">
@@ -11241,18 +11187,18 @@
         <v>46</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
         <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
@@ -11279,7 +11225,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" s="2">
         <v>0</v>
@@ -11295,18 +11241,18 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF3F26B5-E571-48A5-98D0-6FA8C2E9C782}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AD4E396-51FC-4715-A93B-2594F6C9B990}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.4">
@@ -11314,18 +11260,18 @@
         <v>46</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
         <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
@@ -11341,7 +11287,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" s="2">
         <v>0</v>
@@ -11357,18 +11303,18 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C7A977D-83BB-402A-91E4-D23BB940CE9A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{814E1678-E537-4BC9-845E-1FD1B554C445}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="31.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.4">
@@ -11376,18 +11322,18 @@
         <v>46</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
         <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
@@ -11403,7 +11349,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" s="2">
         <v>0</v>
@@ -11419,35 +11365,35 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F6ECF98-E59A-4847-852F-4E406C5B81F9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{443E9EF1-897F-44EC-8319-B373F4839F31}">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="6.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="19.5" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A3" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" t="s">
         <v>63</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>64</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>65</v>
-      </c>
-      <c r="E3" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.4">
@@ -11469,7 +11415,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A5" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" s="5">
         <v>0</v>

</xml_diff>